<commit_message>
Fix video thumbnails and ensure fallback persistence
</commit_message>
<xml_diff>
--- a/YouTube_Studio_CMS_Template_Kids_Content.xlsx
+++ b/YouTube_Studio_CMS_Template_Kids_Content.xlsx
@@ -732,7 +732,7 @@
         <v>Educational kids content.</v>
       </c>
       <c r="D3" t="str">
-        <v>https://picsum.photos/seed/1/640/360</v>
+        <v>/thumbnails/2.webp</v>
       </c>
       <c r="E3" t="str">
         <v>https://youtu.be/demo2</v>
@@ -800,7 +800,7 @@
         <v>Educational kids content.</v>
       </c>
       <c r="D4" t="str">
-        <v>https://picsum.photos/seed/2/640/360</v>
+        <v>/thumbnails/3.webp</v>
       </c>
       <c r="E4" t="str">
         <v>https://youtu.be/demo3</v>
@@ -868,7 +868,7 @@
         <v>Educational kids content.</v>
       </c>
       <c r="D5" t="str">
-        <v>https://picsum.photos/seed/3/640/360</v>
+        <v>/thumbnails/4.webp</v>
       </c>
       <c r="E5" t="str">
         <v>https://youtu.be/demo4</v>
@@ -936,7 +936,7 @@
         <v>Educational kids content.</v>
       </c>
       <c r="D6" t="str">
-        <v>https://picsum.photos/seed/4/640/360</v>
+        <v>/thumbnails/5.webp</v>
       </c>
       <c r="E6" t="str">
         <v>https://youtu.be/demo5</v>
@@ -1004,7 +1004,7 @@
         <v>Educational kids content.</v>
       </c>
       <c r="D7" t="str">
-        <v>https://picsum.photos/seed/5/640/360</v>
+        <v>/thumbnails/6.webp</v>
       </c>
       <c r="E7" t="str">
         <v>https://youtu.be/demo6</v>
@@ -1072,7 +1072,7 @@
         <v>Educational kids content.</v>
       </c>
       <c r="D8" t="str">
-        <v>https://picsum.photos/seed/6/640/360</v>
+        <v>/thumbnails/7.webp</v>
       </c>
       <c r="E8" t="str">
         <v>https://youtu.be/demo7</v>
@@ -1140,7 +1140,7 @@
         <v>Educational kids content.</v>
       </c>
       <c r="D9" t="str">
-        <v>https://picsum.photos/seed/7/640/360</v>
+        <v>/thumbnails/1.webp</v>
       </c>
       <c r="E9" t="str">
         <v>https://youtu.be/demo8</v>
@@ -1208,7 +1208,7 @@
         <v>Educational kids content.</v>
       </c>
       <c r="D10" t="str">
-        <v>https://picsum.photos/seed/8/640/360</v>
+        <v>/thumbnails/2.webp</v>
       </c>
       <c r="E10" t="str">
         <v>https://youtu.be/demo9</v>
@@ -1276,7 +1276,7 @@
         <v>Educational kids content.</v>
       </c>
       <c r="D11" t="str">
-        <v>https://picsum.photos/seed/9/640/360</v>
+        <v>/thumbnails/3.webp</v>
       </c>
       <c r="E11" t="str">
         <v>https://youtu.be/demo10</v>

</xml_diff>

<commit_message>
Update video & channel metrics, date range, and sync Excel CMS template
</commit_message>
<xml_diff>
--- a/YouTube_Studio_CMS_Template_Kids_Content.xlsx
+++ b/YouTube_Studio_CMS_Template_Kids_Content.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:J14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,37 +415,28 @@
         <v>Handle</v>
       </c>
       <c r="C1" t="str">
-        <v>Avatar URL</v>
+        <v>Subscribers</v>
       </c>
       <c r="D1" t="str">
-        <v>Banner URL</v>
+        <v>Lifetime Views</v>
       </c>
       <c r="E1" t="str">
-        <v>Subscribers</v>
+        <v>Monthly Revenue</v>
       </c>
       <c r="F1" t="str">
-        <v>Lifetime Views</v>
+        <v>Average RPM</v>
       </c>
       <c r="G1" t="str">
+        <v>Average CPM</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Country</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="J1" t="str">
         <v>Total Watch Time (hrs)</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Monthly Revenue</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Average RPM</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Average CPM</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Country</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Created Date</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Description</v>
       </c>
     </row>
     <row r="2">
@@ -455,26 +446,29 @@
       <c r="B2" t="str">
         <v>@kidstoons</v>
       </c>
+      <c r="C2">
+        <v>134721</v>
+      </c>
+      <c r="D2">
+        <v>21450000</v>
+      </c>
       <c r="E2">
-        <v>401842</v>
+        <v>2118647.13</v>
       </c>
       <c r="F2">
-        <v>18684271</v>
-      </c>
-      <c r="H2">
-        <v>18743</v>
-      </c>
-      <c r="I2">
         <v>33.64</v>
       </c>
+      <c r="G2">
+        <v>58</v>
+      </c>
+      <c r="H2" t="str">
+        <v>United States</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Fun educational cartoons, nursery rhymes, ABCs, counting, colors, and learning videos for toddlers and preschoolers.</v>
+      </c>
       <c r="J2">
-        <v>57.82</v>
-      </c>
-      <c r="K2" t="str">
-        <v>United States</v>
-      </c>
-      <c r="M2" t="str">
-        <v>Fun educational cartoons, nursery rhymes, ABCs, counting, colors, and learning videos for toddlers and preschoolers.</v>
+        <v>47380</v>
       </c>
     </row>
     <row r="3">
@@ -506,7 +500,7 @@
         <v>Subscribers</v>
       </c>
       <c r="B6">
-        <v>18742391</v>
+        <v>134721</v>
       </c>
     </row>
     <row r="7">
@@ -514,7 +508,7 @@
         <v>Lifetime Views</v>
       </c>
       <c r="B7">
-        <v>6840000000</v>
+        <v>21450000</v>
       </c>
     </row>
     <row r="8">
@@ -522,7 +516,7 @@
         <v>Total Watch Time (hrs)</v>
       </c>
       <c r="B8">
-        <v>12800000</v>
+        <v>47380</v>
       </c>
     </row>
     <row r="9">
@@ -530,7 +524,7 @@
         <v>Monthly Revenue</v>
       </c>
       <c r="B9">
-        <v>486247</v>
+        <v>2118647.13</v>
       </c>
     </row>
     <row r="10">
@@ -574,9 +568,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -676,7 +669,7 @@
         <v>Public</v>
       </c>
       <c r="H2">
-        <v>274365</v>
+        <v>240564</v>
       </c>
       <c r="I2">
         <v>72356</v>
@@ -691,25 +684,25 @@
         <v>8.9</v>
       </c>
       <c r="M2">
-        <v>435.066426</v>
+        <v>427.3865</v>
       </c>
       <c r="N2">
-        <v>791.03</v>
+        <v>58.65</v>
       </c>
       <c r="O2">
-        <v>52346</v>
+        <v>51490</v>
       </c>
       <c r="P2" t="str">
         <v>11:27</v>
       </c>
       <c r="Q2">
-        <v>4946</v>
+        <v>4281</v>
       </c>
       <c r="R2">
-        <v>-125</v>
+        <v>0</v>
       </c>
       <c r="S2">
-        <v>119367</v>
+        <v>102813.79</v>
       </c>
       <c r="T2" t="str">
         <v>Education</v>
@@ -2899,7 +2892,7 @@
         <v>286000</v>
       </c>
       <c r="C2">
-        <v>18742631</v>
+        <v>134721</v>
       </c>
       <c r="D2">
         <v>41470</v>
@@ -2913,7 +2906,7 @@
         <v>304000</v>
       </c>
       <c r="C3">
-        <v>18742751</v>
+        <v>134721</v>
       </c>
       <c r="D3">
         <v>44080</v>
@@ -2927,7 +2920,7 @@
         <v>322000</v>
       </c>
       <c r="C4">
-        <v>18742871</v>
+        <v>134721</v>
       </c>
       <c r="D4">
         <v>46690</v>
@@ -2941,7 +2934,7 @@
         <v>340000</v>
       </c>
       <c r="C5">
-        <v>18742991</v>
+        <v>134721</v>
       </c>
       <c r="D5">
         <v>49300</v>
@@ -2955,7 +2948,7 @@
         <v>358000</v>
       </c>
       <c r="C6">
-        <v>18743111</v>
+        <v>134721</v>
       </c>
       <c r="D6">
         <v>51910</v>
@@ -2969,14 +2962,13 @@
         <v>376000</v>
       </c>
       <c r="C7">
-        <v>18743231</v>
+        <v>134721</v>
       </c>
       <c r="D7">
         <v>54520</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Update video and channel analytics metrics and date range to Sep 19 - Oct 16, 2026
</commit_message>
<xml_diff>
--- a/YouTube_Studio_CMS_Template_Kids_Content.xlsx
+++ b/YouTube_Studio_CMS_Template_Kids_Content.xlsx
@@ -447,13 +447,13 @@
         <v>@kidstoons</v>
       </c>
       <c r="C2">
-        <v>134721</v>
+        <v>138746</v>
       </c>
       <c r="D2">
         <v>21450000</v>
       </c>
       <c r="E2">
-        <v>2118647.13</v>
+        <v>2123743.76</v>
       </c>
       <c r="F2">
         <v>33.64</v>
@@ -468,7 +468,7 @@
         <v>Fun educational cartoons, nursery rhymes, ABCs, counting, colors, and learning videos for toddlers and preschoolers.</v>
       </c>
       <c r="J2">
-        <v>47380</v>
+        <v>49190</v>
       </c>
     </row>
     <row r="3">
@@ -500,7 +500,7 @@
         <v>Subscribers</v>
       </c>
       <c r="B6">
-        <v>134721</v>
+        <v>138746</v>
       </c>
     </row>
     <row r="7">
@@ -516,7 +516,7 @@
         <v>Total Watch Time (hrs)</v>
       </c>
       <c r="B8">
-        <v>47380</v>
+        <v>49190</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         <v>Monthly Revenue</v>
       </c>
       <c r="B9">
-        <v>2118647.13</v>
+        <v>2123743.76</v>
       </c>
     </row>
     <row r="10">
@@ -669,7 +669,7 @@
         <v>Public</v>
       </c>
       <c r="H2">
-        <v>240564</v>
+        <v>243591</v>
       </c>
       <c r="I2">
         <v>72356</v>
@@ -684,25 +684,25 @@
         <v>8.9</v>
       </c>
       <c r="M2">
-        <v>427.3865</v>
+        <v>427.3866</v>
       </c>
       <c r="N2">
         <v>58.65</v>
       </c>
       <c r="O2">
-        <v>51490</v>
+        <v>52140</v>
       </c>
       <c r="P2" t="str">
         <v>11:27</v>
       </c>
       <c r="Q2">
-        <v>4281</v>
+        <v>4157</v>
       </c>
       <c r="R2">
         <v>0</v>
       </c>
       <c r="S2">
-        <v>102813.79</v>
+        <v>104107.53</v>
       </c>
       <c r="T2" t="str">
         <v>Education</v>
@@ -2892,7 +2892,7 @@
         <v>286000</v>
       </c>
       <c r="C2">
-        <v>134721</v>
+        <v>138746</v>
       </c>
       <c r="D2">
         <v>41470</v>
@@ -2906,7 +2906,7 @@
         <v>304000</v>
       </c>
       <c r="C3">
-        <v>134721</v>
+        <v>138746</v>
       </c>
       <c r="D3">
         <v>44080</v>
@@ -2920,7 +2920,7 @@
         <v>322000</v>
       </c>
       <c r="C4">
-        <v>134721</v>
+        <v>138746</v>
       </c>
       <c r="D4">
         <v>46690</v>
@@ -2934,7 +2934,7 @@
         <v>340000</v>
       </c>
       <c r="C5">
-        <v>134721</v>
+        <v>138746</v>
       </c>
       <c r="D5">
         <v>49300</v>
@@ -2948,7 +2948,7 @@
         <v>358000</v>
       </c>
       <c r="C6">
-        <v>134721</v>
+        <v>138746</v>
       </c>
       <c r="D6">
         <v>51910</v>
@@ -2962,7 +2962,7 @@
         <v>376000</v>
       </c>
       <c r="C7">
-        <v>134721</v>
+        <v>138746</v>
       </c>
       <c r="D7">
         <v>54520</v>

</xml_diff>

<commit_message>
Update channel and top video metrics for Sep 26 - Oct 23 date range
</commit_message>
<xml_diff>
--- a/YouTube_Studio_CMS_Template_Kids_Content.xlsx
+++ b/YouTube_Studio_CMS_Template_Kids_Content.xlsx
@@ -447,13 +447,13 @@
         <v>@kidstoons</v>
       </c>
       <c r="C2">
-        <v>138746</v>
+        <v>141578</v>
       </c>
       <c r="D2">
         <v>21450000</v>
       </c>
       <c r="E2">
-        <v>2123743.76</v>
+        <v>2129374.37</v>
       </c>
       <c r="F2">
         <v>33.64</v>
@@ -468,7 +468,7 @@
         <v>Fun educational cartoons, nursery rhymes, ABCs, counting, colors, and learning videos for toddlers and preschoolers.</v>
       </c>
       <c r="J2">
-        <v>49190</v>
+        <v>55710</v>
       </c>
     </row>
     <row r="3">
@@ -669,7 +669,7 @@
         <v>Public</v>
       </c>
       <c r="H2">
-        <v>243591</v>
+        <v>246809</v>
       </c>
       <c r="I2">
         <v>72356</v>
@@ -684,25 +684,25 @@
         <v>8.9</v>
       </c>
       <c r="M2">
-        <v>427.3866</v>
+        <v>427.3853</v>
       </c>
       <c r="N2">
         <v>58.65</v>
       </c>
       <c r="O2">
-        <v>52140</v>
+        <v>52830</v>
       </c>
       <c r="P2" t="str">
         <v>11:27</v>
       </c>
       <c r="Q2">
-        <v>4157</v>
+        <v>4015</v>
       </c>
       <c r="R2">
         <v>0</v>
       </c>
       <c r="S2">
-        <v>104107.53</v>
+        <v>105482.56</v>
       </c>
       <c r="T2" t="str">
         <v>Education</v>
@@ -2892,7 +2892,7 @@
         <v>286000</v>
       </c>
       <c r="C2">
-        <v>138746</v>
+        <v>141578</v>
       </c>
       <c r="D2">
         <v>41470</v>
@@ -2906,7 +2906,7 @@
         <v>304000</v>
       </c>
       <c r="C3">
-        <v>138746</v>
+        <v>141578</v>
       </c>
       <c r="D3">
         <v>44080</v>
@@ -2920,7 +2920,7 @@
         <v>322000</v>
       </c>
       <c r="C4">
-        <v>138746</v>
+        <v>141578</v>
       </c>
       <c r="D4">
         <v>46690</v>
@@ -2934,7 +2934,7 @@
         <v>340000</v>
       </c>
       <c r="C5">
-        <v>138746</v>
+        <v>141578</v>
       </c>
       <c r="D5">
         <v>49300</v>
@@ -2948,7 +2948,7 @@
         <v>358000</v>
       </c>
       <c r="C6">
-        <v>138746</v>
+        <v>141578</v>
       </c>
       <c r="D6">
         <v>51910</v>
@@ -2962,7 +2962,7 @@
         <v>376000</v>
       </c>
       <c r="C7">
-        <v>138746</v>
+        <v>141578</v>
       </c>
       <c r="D7">
         <v>54520</v>

</xml_diff>